<commit_message>
update - evaluate v2
</commit_message>
<xml_diff>
--- a/evaluation/evaluation_labels_only.xlsx
+++ b/evaluation/evaluation_labels_only.xlsx
@@ -2030,7 +2030,7 @@
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="138">
       <c r="A24" s="3" t="s">
         <v>124</v>
       </c>
@@ -2065,7 +2065,7 @@
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="111.75">
       <c r="A25" s="3" t="s">
         <v>129</v>
       </c>
@@ -2100,7 +2100,7 @@
         <v>78</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="45.75">
       <c r="A26" s="3" t="s">
         <v>134</v>
       </c>
@@ -2135,7 +2135,7 @@
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="111.75">
       <c r="A27" s="3" t="s">
         <v>139</v>
       </c>
@@ -2170,7 +2170,7 @@
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="150.75">
       <c r="A28" s="3" t="s">
         <v>144</v>
       </c>
@@ -2205,7 +2205,7 @@
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="111.75">
       <c r="A29" s="3" t="s">
         <v>149</v>
       </c>
@@ -2240,7 +2240,7 @@
         <v>22</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="111.75">
       <c r="A30" s="3" t="s">
         <v>154</v>
       </c>

</xml_diff>